<commit_message>
updated exp results xlsx files
</commit_message>
<xml_diff>
--- a/Experimental_Results/Protocol-1_15_DF_Detectors_ACC.xlsx
+++ b/Experimental_Results/Protocol-1_15_DF_Detectors_ACC.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DOWNLOADs\Dropbox\PhD-TUBerlin\PUBLICATIONs\2026\WWW2026\Experiments\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WORKSPACE\GIT\MoORD\Experimental_Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{093137D1-C8C6-419D-A06D-04AD7AA1C2E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB99872D-78AA-44CE-BDCA-0CCED65AABDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12552" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -155,6 +155,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.000"/>
+  </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -371,7 +374,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -383,16 +386,40 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -401,56 +428,46 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -744,314 +761,314 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="35.4" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="12"/>
-      <c r="E1" s="13" t="s">
+      <c r="D1" s="14"/>
+      <c r="E1" s="19" t="s">
         <v>3</v>
       </c>
       <c r="F1" s="4"/>
     </row>
     <row r="2" spans="1:6" ht="18.3" thickTop="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A2" s="7"/>
-      <c r="B2" s="10"/>
+      <c r="A2" s="16"/>
+      <c r="B2" s="18"/>
       <c r="C2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="20" t="s">
+      <c r="D2" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="6"/>
+      <c r="E2" s="20"/>
       <c r="F2" s="4"/>
     </row>
     <row r="3" spans="1:6" ht="20.05" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="18">
+      <c r="C3" s="21">
         <v>0.59499999999999997</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D3" s="22">
         <v>0.53200000000000003</v>
       </c>
-      <c r="E3" s="18">
-        <f>(C3+D3)/2</f>
+      <c r="E3" s="21">
+        <f t="shared" ref="E3:E17" si="0">(C3+D3)/2</f>
         <v>0.5635</v>
       </c>
       <c r="F3" s="4"/>
     </row>
     <row r="4" spans="1:6" ht="20.05" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A4" s="16" t="s">
+      <c r="A4" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="15">
+      <c r="C4" s="23">
         <v>0.53259999999999996</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="24">
         <v>0.49099999999999999</v>
       </c>
-      <c r="E4" s="15">
-        <f>(C4+D4)/2</f>
+      <c r="E4" s="23">
+        <f t="shared" si="0"/>
         <v>0.51180000000000003</v>
       </c>
       <c r="F4" s="4"/>
     </row>
     <row r="5" spans="1:6" ht="20.05" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="14">
+      <c r="C5" s="25">
         <v>0.46100000000000002</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="24">
         <v>0.28799999999999998</v>
       </c>
-      <c r="E5" s="16">
-        <f>(C5+D5)/2</f>
+      <c r="E5" s="26">
+        <f t="shared" si="0"/>
         <v>0.3745</v>
       </c>
       <c r="F5" s="4"/>
     </row>
     <row r="6" spans="1:6" ht="20.05" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A6" s="17" t="s">
+      <c r="A6" s="8" t="s">
         <v>11</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="18">
+      <c r="C6" s="21">
         <v>0.45</v>
       </c>
-      <c r="D6" s="21">
+      <c r="D6" s="27">
         <v>0.27900000000000003</v>
       </c>
-      <c r="E6" s="16">
-        <f>(C6+D6)/2</f>
+      <c r="E6" s="26">
+        <f t="shared" si="0"/>
         <v>0.36450000000000005</v>
       </c>
       <c r="F6" s="4"/>
     </row>
     <row r="7" spans="1:6" ht="20.05" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="14">
+      <c r="C7" s="25">
         <v>0.65500000000000003</v>
       </c>
-      <c r="D7" s="22">
+      <c r="D7" s="28">
         <v>0.6</v>
       </c>
-      <c r="E7" s="14">
-        <f>(C7+D7)/2</f>
+      <c r="E7" s="25">
+        <f t="shared" si="0"/>
         <v>0.62749999999999995</v>
       </c>
       <c r="F7" s="4"/>
     </row>
     <row r="8" spans="1:6" ht="20.05" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="16" t="s">
+      <c r="B8" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="18">
+      <c r="C8" s="21">
         <v>0.66</v>
       </c>
-      <c r="D8" s="21">
+      <c r="D8" s="27">
         <v>0.58199999999999996</v>
       </c>
-      <c r="E8" s="19">
-        <f>(C8+D8)/2</f>
+      <c r="E8" s="29">
+        <f t="shared" si="0"/>
         <v>0.621</v>
       </c>
       <c r="F8" s="4"/>
     </row>
     <row r="9" spans="1:6" ht="20.05" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="16" t="s">
+      <c r="B9" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="15">
+      <c r="C9" s="23">
         <v>0.52100000000000002</v>
       </c>
-      <c r="D9" s="21">
+      <c r="D9" s="27">
         <v>0.496</v>
       </c>
-      <c r="E9" s="15">
-        <f>(C9+D9)/2</f>
+      <c r="E9" s="23">
+        <f t="shared" si="0"/>
         <v>0.50849999999999995</v>
       </c>
       <c r="F9" s="4"/>
     </row>
     <row r="10" spans="1:6" ht="20.05" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="18">
+      <c r="C10" s="21">
         <v>0.41899999999999998</v>
       </c>
-      <c r="D10" s="21">
+      <c r="D10" s="27">
         <v>0.38800000000000001</v>
       </c>
-      <c r="E10" s="18">
-        <f>(C10+D10)/2</f>
+      <c r="E10" s="21">
+        <f t="shared" si="0"/>
         <v>0.40349999999999997</v>
       </c>
       <c r="F10" s="4"/>
     </row>
     <row r="11" spans="1:6" ht="20.05" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A11" s="17" t="s">
+      <c r="A11" s="8" t="s">
         <v>21</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="18">
+      <c r="C11" s="21">
         <v>0.68600000000000005</v>
       </c>
-      <c r="D11" s="21">
+      <c r="D11" s="27">
         <v>0.65</v>
       </c>
-      <c r="E11" s="18">
-        <f>(C11+D11)/2</f>
+      <c r="E11" s="21">
+        <f t="shared" si="0"/>
         <v>0.66800000000000004</v>
       </c>
       <c r="F11" s="4"/>
     </row>
     <row r="12" spans="1:6" ht="20.05" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A12" s="16" t="s">
+      <c r="A12" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="C12" s="1">
+      <c r="C12" s="22">
         <v>0.63600000000000001</v>
       </c>
-      <c r="D12" s="21">
+      <c r="D12" s="27">
         <v>0.54100000000000004</v>
       </c>
-      <c r="E12" s="15">
-        <f>(C12+D12)/2</f>
+      <c r="E12" s="23">
+        <f t="shared" si="0"/>
         <v>0.58850000000000002</v>
       </c>
       <c r="F12" s="4"/>
     </row>
     <row r="13" spans="1:6" ht="20.05" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A13" s="16" t="s">
+      <c r="A13" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="15" t="s">
+      <c r="B13" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C13" s="18">
+      <c r="C13" s="21">
         <v>0.45800000000000002</v>
       </c>
-      <c r="D13" s="21">
+      <c r="D13" s="27">
         <v>0.38800000000000001</v>
       </c>
-      <c r="E13" s="19">
-        <f>(C13+D13)/2</f>
+      <c r="E13" s="29">
+        <f t="shared" si="0"/>
         <v>0.42300000000000004</v>
       </c>
       <c r="F13" s="4"/>
     </row>
     <row r="14" spans="1:6" ht="20.05" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A14" s="16" t="s">
+      <c r="A14" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="C14" s="1">
+      <c r="C14" s="22">
         <v>0.63100000000000001</v>
       </c>
-      <c r="D14" s="21">
+      <c r="D14" s="27">
         <v>0.60199999999999998</v>
       </c>
-      <c r="E14" s="19">
-        <f>(C14+D14)/2</f>
+      <c r="E14" s="29">
+        <f t="shared" si="0"/>
         <v>0.61650000000000005</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="20.05" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A15" s="16" t="s">
+      <c r="A15" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="25" t="s">
+      <c r="B15" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="C15" s="18">
+      <c r="C15" s="21">
         <v>0.72299999999999998</v>
       </c>
-      <c r="D15" s="21">
+      <c r="D15" s="27">
         <v>0.71099999999999997</v>
       </c>
-      <c r="E15" s="18">
-        <f>(C15+D15)/2</f>
+      <c r="E15" s="21">
+        <f t="shared" si="0"/>
         <v>0.71699999999999997</v>
       </c>
       <c r="F15" s="4"/>
     </row>
     <row r="16" spans="1:6" ht="20.05" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A16" s="16" t="s">
+      <c r="A16" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B16" s="16" t="s">
+      <c r="B16" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C16" s="18">
+      <c r="C16" s="21">
         <v>0.57699999999999996</v>
       </c>
-      <c r="D16" s="21">
+      <c r="D16" s="27">
         <v>0.53500000000000003</v>
       </c>
-      <c r="E16" s="15">
-        <f>(C16+D16)/2</f>
+      <c r="E16" s="23">
+        <f t="shared" si="0"/>
         <v>0.55600000000000005</v>
       </c>
       <c r="F16" s="4"/>
     </row>
     <row r="17" spans="1:6" ht="20.05" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A17" s="23" t="s">
+      <c r="A17" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="B17" s="16" t="s">
+      <c r="B17" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="C17" s="26">
+      <c r="C17" s="30">
         <v>0.80800000000000005</v>
       </c>
-      <c r="D17" s="27">
-        <v>0.76300000000000001</v>
-      </c>
-      <c r="E17" s="28">
+      <c r="D17" s="31">
+        <v>0.76600000000000001</v>
+      </c>
+      <c r="E17" s="32">
         <f>(C17+D17)/2</f>
-        <v>0.78550000000000009</v>
+        <v>0.78700000000000003</v>
       </c>
       <c r="F17" s="4"/>
     </row>
@@ -1061,7 +1078,6 @@
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
       <c r="E18" s="3"/>
-      <c r="F18" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>